<commit_message>
Restore Kakamega's original workbook values
Kakamega's inputs match main again: the Phase 1 routing values added earlier are
removed (blank cells), so Kakamega runs the original model. The shared mortality
constants p_mat_death_facility_baseline and RR_MM_l23_vs_l4 are blank, so their
fallbacks apply. tests/test_kakamega_original.py now passes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SDR Parameters.xlsx
+++ b/SDR Parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/meibinchen/Documents/GitHub/SDR-Dashboard-2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08450A9A-39AD-A049-916A-AF08485D6E51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C47B848-8556-8F48-9AFE-A592ED0B16A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="21420" yWindow="600" windowWidth="16980" windowHeight="21000" firstSheet="14" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="23600" yWindow="600" windowWidth="12860" windowHeight="21000" firstSheet="13" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="30" r:id="rId1"/>
@@ -9197,9 +9197,7 @@
       <c r="A37" s="5" t="s">
         <v>1281</v>
       </c>
-      <c r="B37" s="5">
-        <v>2.85382E-3</v>
-      </c>
+      <c r="B37" s="5"/>
       <c r="C37" s="5"/>
       <c r="D37" s="5"/>
       <c r="E37" s="5"/>
@@ -9210,9 +9208,7 @@
       <c r="A38" s="5" t="s">
         <v>1282</v>
       </c>
-      <c r="B38" s="5">
-        <v>2.2376019999999999</v>
-      </c>
+      <c r="B38" s="5"/>
       <c r="C38" s="5"/>
       <c r="D38" s="5"/>
       <c r="E38" s="5"/>
@@ -12251,7 +12247,7 @@
         <v>433</v>
       </c>
       <c r="C14" s="5">
-        <v>0.73350000000000004</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="D14" s="5">
         <v>0.49399999999999999</v>
@@ -12852,7 +12848,7 @@
         <v>433</v>
       </c>
       <c r="C34" s="5">
-        <v>4550</v>
+        <v>2989.08</v>
       </c>
       <c r="D34" s="5"/>
       <c r="E34" s="5"/>
@@ -15630,7 +15626,7 @@
         <v>433</v>
       </c>
       <c r="C2" s="5">
-        <v>4.7899999999999998E-2</v>
+        <v>0.70599999999999996</v>
       </c>
       <c r="D2" s="5"/>
       <c r="E2" s="5" t="s">
@@ -15773,7 +15769,7 @@
         <v>433</v>
       </c>
       <c r="C10" s="5">
-        <v>6.93E-2</v>
+        <v>0.16919999999999999</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="5" t="s">
@@ -16079,7 +16075,7 @@
         <v>433</v>
       </c>
       <c r="C26" s="5">
-        <v>0.72130000000000005</v>
+        <v>0.82509999999999994</v>
       </c>
       <c r="D26" s="5"/>
       <c r="E26" s="5" t="s">
@@ -16154,7 +16150,7 @@
         <v>433</v>
       </c>
       <c r="C30" s="5">
-        <v>6.157E-2</v>
+        <v>6.4199999999999993E-2</v>
       </c>
       <c r="D30" s="5"/>
       <c r="E30" s="5" t="s">
@@ -16229,7 +16225,7 @@
         <v>433</v>
       </c>
       <c r="C34" s="5">
-        <v>0.71870000000000001</v>
+        <v>0.77990000000000004</v>
       </c>
       <c r="D34" s="5"/>
       <c r="E34" s="5" t="s">
@@ -16463,7 +16459,7 @@
         <v>433</v>
       </c>
       <c r="C46" s="5">
-        <v>2.07E-2</v>
+        <v>1.7600000000000001E-2</v>
       </c>
       <c r="D46" s="5"/>
       <c r="E46" s="5" t="s">
@@ -16538,7 +16534,7 @@
         <v>433</v>
       </c>
       <c r="C50" s="5">
-        <v>2.1020087757315786E-2</v>
+        <v>1.6400000000000001E-2</v>
       </c>
       <c r="D50" s="5"/>
       <c r="E50" s="5" t="s">
@@ -16613,7 +16609,7 @@
         <v>433</v>
       </c>
       <c r="C54" s="5">
-        <v>2.7000000000000001E-3</v>
+        <v>1.9099999999999999E-2</v>
       </c>
       <c r="D54" s="5"/>
       <c r="E54" s="5" t="s">
@@ -16688,7 +16684,7 @@
         <v>433</v>
       </c>
       <c r="C58" s="5">
-        <v>1.542</v>
+        <v>0.79820000000000002</v>
       </c>
       <c r="D58" s="5"/>
       <c r="E58" s="5" t="s">
@@ -16918,7 +16914,7 @@
         <v>433</v>
       </c>
       <c r="C71" s="5">
-        <v>7.5249999999999997E-2</v>
+        <v>5.6800000000000003E-2</v>
       </c>
       <c r="D71" s="5">
         <v>1</v>
@@ -16938,7 +16934,7 @@
         <v>433</v>
       </c>
       <c r="C72" s="5">
-        <v>5.11E-2</v>
+        <v>0.1215</v>
       </c>
       <c r="D72" s="5">
         <v>2</v>
@@ -18205,7 +18201,7 @@
         <v>433</v>
       </c>
       <c r="C142" s="5">
-        <v>8.2949999999999996E-2</v>
+        <v>5.0099999999999999E-2</v>
       </c>
       <c r="D142" s="5"/>
       <c r="E142" s="5" t="s">
@@ -18397,7 +18393,7 @@
         <v>433</v>
       </c>
       <c r="C154" s="5">
-        <v>87.135999999999996</v>
+        <v>0.80948500000000001</v>
       </c>
       <c r="D154" s="5"/>
       <c r="E154" s="5" t="s">
@@ -18475,7 +18471,7 @@
         <v>433</v>
       </c>
       <c r="C158" s="5">
-        <v>96.034000000000006</v>
+        <v>0.74235799999999996</v>
       </c>
       <c r="D158" s="5"/>
       <c r="E158" s="5" t="s">
@@ -18553,7 +18549,7 @@
         <v>433</v>
       </c>
       <c r="C162" s="5">
-        <v>90</v>
+        <v>0.9</v>
       </c>
       <c r="D162" s="5"/>
       <c r="E162" s="5" t="s">
@@ -18621,9 +18617,7 @@
       <c r="B166" s="5" t="s">
         <v>433</v>
       </c>
-      <c r="C166" s="2">
-        <v>1.45</v>
-      </c>
+      <c r="C166" s="2"/>
       <c r="D166" s="2"/>
       <c r="E166" s="2"/>
       <c r="G166" s="2"/>
@@ -18686,9 +18680,7 @@
       <c r="B170" s="5" t="s">
         <v>433</v>
       </c>
-      <c r="C170" s="2">
-        <v>8.3280000000000007E-2</v>
-      </c>
+      <c r="C170" s="2"/>
       <c r="D170" s="2"/>
       <c r="E170" s="2"/>
       <c r="G170" s="2"/>
@@ -18751,9 +18743,7 @@
       <c r="B174" s="2" t="s">
         <v>433</v>
       </c>
-      <c r="C174" s="2">
-        <v>0.35599999999999998</v>
-      </c>
+      <c r="C174" s="2"/>
       <c r="D174" s="2"/>
       <c r="E174" s="2" t="s">
         <v>1228</v>
@@ -18827,9 +18817,7 @@
       <c r="B178" s="2" t="s">
         <v>433</v>
       </c>
-      <c r="C178" s="2">
-        <v>2</v>
-      </c>
+      <c r="C178" s="2"/>
       <c r="D178" s="2"/>
       <c r="E178" s="2" t="s">
         <v>1231</v>
@@ -18903,9 +18891,7 @@
       <c r="B182" s="2" t="s">
         <v>433</v>
       </c>
-      <c r="C182" s="2">
-        <v>42.996000000000002</v>
-      </c>
+      <c r="C182" s="2"/>
       <c r="D182" s="2"/>
       <c r="E182" t="s">
         <v>1280</v>

</xml_diff>

<commit_message>
Replace PULSE: PROMPTS registration and health-worker knowledge (Ivers 2026); FQA no longer reaches home births in Kisii, Makueni and Mombasa
</commit_message>
<xml_diff>
--- a/SDR Parameters.xlsx
+++ b/SDR Parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/meibinchen/Documents/GitHub/SDR-Dashboard-2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C47B848-8556-8F48-9AFE-A592ED0B16A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ACC397B-8DF5-554D-859C-1AD1AC141B71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23600" yWindow="600" windowWidth="12860" windowHeight="21000" firstSheet="13" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="21820" yWindow="600" windowWidth="14640" windowHeight="21000" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="30" r:id="rId1"/>
@@ -99,7 +99,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12367" uniqueCount="1300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12375" uniqueCount="1302">
   <si>
     <t xml:space="preserve">Append table last refreshed: </t>
   </si>
@@ -4251,6 +4251,12 @@
   <si>
     <t>Stage 6 candidate (shared; pooled KHIS L2/3 and internal-L4 MMR)</t>
   </si>
+  <si>
+    <t>pulse_or_prompts_registration</t>
+  </si>
+  <si>
+    <t>pulse_performance_improve</t>
+  </si>
 </sst>
 </file>
 
@@ -4260,7 +4266,7 @@
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="33" x14ac:knownFonts="1">
+  <fonts count="34" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -4475,6 +4481,12 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color rgb="FF616161"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -4854,7 +4866,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="160">
+  <cellXfs count="162">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -5125,6 +5137,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -7965,8 +7981,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF08000000}" name="Table3" displayName="Table3" ref="A1:L59" totalsRowShown="0" dataDxfId="109">
-  <autoFilter ref="A1:L59" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF08000000}" name="Table3" displayName="Table3" ref="A1:L61" totalsRowShown="0" dataDxfId="109">
+  <autoFilter ref="A1:L61" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0800-000001000000}" name="parameter_name" dataDxfId="108"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0800-000002000000}" name="value" dataDxfId="107"/>
@@ -66869,7 +66885,7 @@
   <sheetPr>
     <tabColor theme="4"/>
   </sheetPr>
-  <dimension ref="A1:O59"/>
+  <dimension ref="A1:O61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="18.33203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -68609,10 +68625,10 @@
         <v>292</v>
       </c>
       <c r="G59" s="126"/>
-      <c r="H59" s="126" t="s">
+      <c r="H59" s="111" t="s">
         <v>233</v>
       </c>
-      <c r="I59" s="126" t="s">
+      <c r="I59" s="111" t="s">
         <v>233</v>
       </c>
       <c r="J59" s="55" t="s">
@@ -68622,6 +68638,62 @@
       <c r="L59" s="113" t="s">
         <v>321</v>
       </c>
+    </row>
+    <row r="60" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+      <c r="A60" s="55" t="s">
+        <v>1300</v>
+      </c>
+      <c r="B60" s="161">
+        <v>1.47</v>
+      </c>
+      <c r="C60" s="55">
+        <v>1.31</v>
+      </c>
+      <c r="D60" s="55">
+        <v>1.64</v>
+      </c>
+      <c r="E60" s="55"/>
+      <c r="F60" s="111" t="s">
+        <v>228</v>
+      </c>
+      <c r="G60" s="126"/>
+      <c r="H60" s="111" t="s">
+        <v>233</v>
+      </c>
+      <c r="I60" s="111" t="s">
+        <v>233</v>
+      </c>
+      <c r="J60" s="55"/>
+      <c r="K60" s="55"/>
+      <c r="L60" s="160"/>
+    </row>
+    <row r="61" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+      <c r="A61" s="55" t="s">
+        <v>1301</v>
+      </c>
+      <c r="B61" s="161">
+        <v>6.2E-2</v>
+      </c>
+      <c r="C61" s="161">
+        <v>4.1000000000000002E-2</v>
+      </c>
+      <c r="D61" s="161">
+        <v>8.2000000000000003E-2</v>
+      </c>
+      <c r="E61" s="55"/>
+      <c r="F61" s="111" t="s">
+        <v>228</v>
+      </c>
+      <c r="G61" s="126"/>
+      <c r="H61" s="111" t="s">
+        <v>233</v>
+      </c>
+      <c r="I61" s="111" t="s">
+        <v>233</v>
+      </c>
+      <c r="J61" s="55"/>
+      <c r="K61" s="55"/>
+      <c r="L61" s="160"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>